<commit_message>
Update menu, product photos, weights and mobile UX
- New product photos (brownies, tea cakes); tea cakes 300 g, Original brownie 500g
- Sheet-driven data layer, 1 kg bundt labels, (contains eggs) note
- Order sheet: Opened in WhatsApp state, quiet copy link
- Add-to-order on home product screens with Added feedback
- Header WhatsApp icon on phones, mobile menu navigation fixes
- Footer Contact opens the dialler; Mylo & Alexa highlighted
- Menu preview shows piece counts; refreshed menu PDF and Excel template

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/menu-data/INdulgence-menu-data.xlsx
+++ b/menu-data/INdulgence-menu-data.xlsx
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A28"/>
+  <dimension ref="A1:A29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -649,33 +649,40 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>•  Photos: type the file name of a picture that is inside the website’s public/products folder (e.g. marble-tea-cake.webp). To use a NEW photo, ask your developer to add the file once; then put its name here. A product with no photo still works.</t>
+          <t>•  The small line under every product’s description (“(contains eggs)”) comes from Content → product_note. To change it for ONE product, type its own text in that product’s “note” cell; type none to hide it for that product (or in Content → product_note to hide it everywhere).</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>•  Menu PDF: paste your Google Drive share link in Settings → menu_pdf_url (Anyone with the link → Viewer). Leave it empty to use the PDF that comes with the website.</t>
+          <t>•  Photos: type the file name of a picture that is inside the website’s public/products folder (e.g. marble-tea-cake.webp). To use a NEW photo, ask your developer to add the file once; then put its name here. A product with no photo still works.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>•  The website re-reads the sheet about every 5 minutes. If the sheet ever can’t be read, the website keeps showing the last good version — it never breaks.</t>
+          <t>•  Menu PDF: paste your Google Drive share link in Settings → menu_pdf_url (Anyone with the link → Viewer). Leave it empty to use the PDF that comes with the website.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>•  Limits: up to 60 products, 8 categories, 3 sizes per product. Very long texts are shortened.</t>
+          <t>•  The website re-reads the sheet about every 5 minutes. If the sheet ever can’t be read, the website keeps showing the last good version — it never breaks.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>•  Limits: up to 60 products, 8 categories, 3 sizes per product. Very long texts are shortened.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>•  This sheet is public to anyone who has the link (they can read it, not edit it). Don’t put anything private in it.</t>
         </is>
@@ -871,7 +878,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1116,49 +1123,66 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>final_headline</t>
+          <t>product_note</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Indulge with intention.</t>
+          <t>(contains eggs)</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Last screen headline.</t>
+          <t>Small line under every product's description. A product can override it with its own 'note' cell (type none to hide it for that product). Type none here to hide it everywhere.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>final_note</t>
+          <t>final_headline</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Freshly prepared to order · 24 hours’ advance notice · 100% payment on confirmation · No COD</t>
+          <t>Indulge with intention.</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Small line under the last headline.</t>
+          <t>Last screen headline.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
+          <t>final_note</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>Freshly prepared to order · 24 hours’ advance notice · 100% payment on confirmation · No COD</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Small line under the last headline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
           <t>footer_note</t>
         </is>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>A portion of every order nourishes stray animals.</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C18" s="7" t="inlineStr">
         <is>
           <t>Footer, bottom right.</t>
         </is>
@@ -1269,7 +1293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1285,6 +1309,7 @@
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
     <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -1353,6 +1378,11 @@
           <t>available</t>
         </is>
       </c>
+      <c r="N1" s="4" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
@@ -1373,17 +1403,17 @@
       <c r="D2" s="6" t="n"/>
       <c r="E2" s="9" t="inlineStr">
         <is>
-          <t>original-indulgence-photo.webp</t>
+          <t>original-indulgence-v2.webp</t>
         </is>
       </c>
       <c r="F2" s="6" t="inlineStr">
         <is>
-          <t>The Original Indulgence brownie with melted chocolate chunks and a crackled top</t>
+          <t>The Original Indulgence brownies stacked beside their iNdulgence box</t>
         </is>
       </c>
       <c r="G2" s="9" t="inlineStr">
         <is>
-          <t>450g / 4pc</t>
+          <t>500g / 4pc</t>
         </is>
       </c>
       <c r="H2" s="11" t="n">
@@ -1398,6 +1428,7 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="N2" s="9" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
@@ -1418,12 +1449,12 @@
       <c r="D3" s="6" t="n"/>
       <c r="E3" s="9" t="inlineStr">
         <is>
-          <t>biscoff-reverie-photo.webp</t>
+          <t>biscoff-reverie-v2.webp</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>The Biscoff Reverie brownie topped with a Lotus Biscoff biscuit over a caramelised Biscoff layer</t>
+          <t>The Biscoff Reverie brownies topped with Lotus Biscoff, beside their iNdulgence box</t>
         </is>
       </c>
       <c r="G3" s="9" t="inlineStr">
@@ -1449,6 +1480,7 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="N3" s="9" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
@@ -1469,12 +1501,12 @@
       <c r="D4" s="6" t="n"/>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>rocher-reserve-photo.webp</t>
+          <t>rocher-reserve-v2.webp</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>The Rocher Reserve brownie crowned with a Ferrero Rocher over a Nutella layer</t>
+          <t>The Rocher Reserve brownies topped with Ferrero Rocher, beside their iNdulgence box</t>
         </is>
       </c>
       <c r="G4" s="9" t="inlineStr">
@@ -1500,6 +1532,7 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="N4" s="9" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -1520,12 +1553,12 @@
       <c r="D5" s="6" t="n"/>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>nutty-elite-photo.webp</t>
+          <t>nutty-elite-v2.webp</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>The Nutty Elite brownie with a pistachio filling and crushed pistachio on top</t>
+          <t>The Nutty Elite pistachio brownies stacked beside their iNdulgence box</t>
         </is>
       </c>
       <c r="G5" s="9" t="inlineStr">
@@ -1551,6 +1584,7 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="N5" s="9" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
@@ -1571,15 +1605,19 @@
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>vanilla-tea-cake.webp</t>
+          <t>vanilla-tea-cake-v2.webp</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>Sliced vanilla tea cake loaf with a golden crust</t>
-        </is>
-      </c>
-      <c r="G6" s="9" t="n"/>
+          <t>Vanilla tea cake slices beside the tea cake box</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>300 g</t>
+        </is>
+      </c>
       <c r="H6" s="11" t="n">
         <v>299</v>
       </c>
@@ -1592,6 +1630,7 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="N6" s="9" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -1612,15 +1651,19 @@
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
-          <t>chocolate-tea-cake.webp</t>
+          <t>chocolate-tea-cake-v2.webp</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>Sliced chocolate tea cake loaf</t>
-        </is>
-      </c>
-      <c r="G7" s="9" t="n"/>
+          <t>Chocolate tea cake slices beside the tea cake box</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>300 g</t>
+        </is>
+      </c>
       <c r="H7" s="11" t="n">
         <v>399</v>
       </c>
@@ -1633,6 +1676,7 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="N7" s="9" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -1653,15 +1697,19 @@
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>marble-tea-cake.webp</t>
+          <t>marble-tea-cake-v2.webp</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>Sliced marble tea cake loaf with chocolate and vanilla swirls</t>
-        </is>
-      </c>
-      <c r="G8" s="9" t="n"/>
+          <t>Marble tea cake slices beside the tea cake box</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>300 g</t>
+        </is>
+      </c>
       <c r="H8" s="11" t="n">
         <v>449</v>
       </c>
@@ -1674,6 +1722,7 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="N8" s="9" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
@@ -1702,7 +1751,11 @@
           <t>Vanilla bundt cake with a golden crust</t>
         </is>
       </c>
-      <c r="G9" s="9" t="n"/>
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>1 kg</t>
+        </is>
+      </c>
       <c r="H9" s="11" t="n">
         <v>699</v>
       </c>
@@ -1715,6 +1768,7 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="N9" s="9" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
@@ -1743,7 +1797,11 @@
           <t>Chocolate bundt cake</t>
         </is>
       </c>
-      <c r="G10" s="9" t="n"/>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>1 kg</t>
+        </is>
+      </c>
       <c r="H10" s="11" t="n">
         <v>799</v>
       </c>
@@ -1756,6 +1814,7 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="N10" s="9" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
@@ -1784,7 +1843,11 @@
           <t>Marble bundt cake with chocolate and vanilla swirls</t>
         </is>
       </c>
-      <c r="G11" s="9" t="n"/>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>1 kg</t>
+        </is>
+      </c>
       <c r="H11" s="11" t="n">
         <v>899</v>
       </c>
@@ -1797,6 +1860,7 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="N11" s="9" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="2">

</xml_diff>